<commit_message>
fix(mobile): a busy login server at app start shows Retry, not the login form
A 429 or 5xx from get-session now sets offline (cookie kept; only 401 signs out). Also: notice target uses the shared request-screen kinds (@kando/contract), notify-me follows its watching prop, hard-coded late-fee and 24 h boundary tests.
</commit_message>
<xml_diff>
--- a/Reports/Assessment-Stage-D-Test-Report.xlsx
+++ b/Reports/Assessment-Stage-D-Test-Report.xlsx
@@ -39908,7 +39908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -40030,7 +40030,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Thrown Responses carry no Cache-Control private,no-store</t>
+          <t>FIXED: thrown Responses and AUTH_BUSY now carry Cache-Control private,no-store</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -40040,12 +40040,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Domain 404, 409 and 400 answers thrown as Responses (app-request.ts:125, admin-request.ts:41) skip the private,no-store header; the item routes changed to the throw path in Task 9. Bodies hold no personal data. No fix commit was on the branch when this report was written. One-line fix proposed by the reviewer.</t>
+          <t>Domain 404, 409 and 400 answers thrown as Responses (app-request.ts:125, admin-request.ts:41) skip the private,no-store header; the item routes changed to the throw path in Task 9. Bodies hold no personal data. Fixed in the final review fix wave (one helper in app-request.ts and admin-request.ts, also on the early 401/403/411/413 answers; an immutable Response is left as it is).</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Later (one line each)</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -40194,7 +40194,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>503 AUTH_BUSY lacks Cache-Control no-store (app-request.ts:129); the test cleanup is not in finally; admin screens show a generic error for 503.</t>
+          <t>(503 AUTH_BUSY no-store: fixed in the final review fix wave.) the test cleanup is not in finally; admin screens show a generic error for 503.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -40244,6 +40244,28 @@
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Owner phone test</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tests added after the final review fix wave</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Final review</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Tests added after the final review fix wave: counts in the combined verification. Covers: busy login on app start gives the Retry screen (use-session), no-store on thrown/busy/early answers (app-request and admin-roles specs), hard-coded late-fee and 24 h boundary numbers (mobile and domain), request-screen kinds list shared via @kando/contract.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Combined verification</t>
         </is>
       </c>
     </row>

</xml_diff>